<commit_message>
chap 11 wiz - time tossed showdown
</commit_message>
<xml_diff>
--- a/docs/final/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/final/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R707fb3d418b94d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rc5954cdef6b347b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rbc8a5fc8ab014553"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Racd8d315d20d4d69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Reb10640b40fd49eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R936babb558b74276"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R0bac06c09d1e4fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rfd298c58804346c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R1f08e155857145d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R49b3288178514f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rff34cd7603c34ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R85d6a3c043f34174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R1efac7caba3e45c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc21296b2b4594ca3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rad6f575b98794c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rba7be72729934091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R75b7b73c3d7d4a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R62ba3e5b5a2a467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Ra8679cb0d7f44d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rbb68f30ac8df41fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R6a4dae1604304b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R882e37f838164e0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R90a4ba6353b343fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rfa634712863941d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R8ca9504e279d4b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R99eecd66598e4de3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5100,10 +5100,8 @@
           <x:t xml:space="preserve">Time-Tossed Showdown</x:t>
         </x:is>
       </x:c>
-      <x:c r="E12" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Placeholder shell — full design/coding required</x:t>
-        </x:is>
+      <x:c r="E12" s="31" t="str">
+        <x:v>Implemented — needs machine playtest/polish</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10225,15 +10223,11 @@
           <x:t xml:space="preserve">start_mode_time_tossed_showdown</x:t>
         </x:is>
       </x:c>
-      <x:c r="F12" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G12" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
+      <x:c r="F12" s="31" t="str">
+        <x:v>Wizard scoring uses Chapter 11 Case Files directly: Master Vine targets = 100K + 20K × collected Case Files; Spider-Men lit-position Jackpots = 250K + 20K × collected Case Files; Master Technician spinner/Star-at-cap = 100K + 20K × collected Case Files + 10K × rooftop upper-target hits. Rooftop setup shots themselves receive only normal/basic upper-playfield scoring.</x:v>
+      </x:c>
+      <x:c r="G12" s="31" t="str">
+        <x:v>Implemented endurance wizard: 3-ball multiball, 20s opening save, 4-ball cap. Each rooftop visit gives 12 setup flips; upper targets build Master Technician value and qualify Spider-Men saucers, while upper-spinner spins light Master Vine shots. Exit selects the lower phase (L Spider-Men / C Master Vine / R Master Technician). Gate opens only for rooftop setup, saucers park for 15s, and the loop repeats until multiball ends. Needs machine playtest/polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -13768,10 +13762,10 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="45" t="str">
-        <x:v>Review remaining functional/provisional mini-wizards; fully design and code the 1 remaining placeholder shell (Time-Tossed Showdown); complete the dedicated Kingpin Final Showdown design/retheme. Who Is the Real Villain? is implemented and needs machine playtest. Wizard Case Files add 20K each to qualifying Jackpot values (max +500K per 1X JP).</x:v>
+        <x:v>Review remaining functional/provisional mini-wizards and complete dedicated Kingpin Final Showdown design/retheme. Time-Tossed Showdown is now implemented and needs machine playtest/polish. Wizard Case Files add 20K each to qualifying Jackpot values (max +500K per 1X JP).</x:v>
       </x:c>
       <x:c r="D14" s="45" t="str">
-        <x:v>In progress</x:v>
+        <x:v>In progress — Time-Tossed implemented; remaining work is review/playtest/polish</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="26" customFormat="1" ht="38" customHeight="1">

</xml_diff>

<commit_message>
park, save timing, ducking
</commit_message>
<xml_diff>
--- a/docs/final/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/final/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -9894,10 +9894,8 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G2" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Approved/coded; needs machine playtest and polish.</x:t>
-        </x:is>
+      <x:c r="G2" s="31" t="str">
+        <x:v>Approved/coded; needs machine playtest and polish. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9929,10 +9927,8 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G3" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Functional provisional implementation; design review and approval still required.</x:t>
-        </x:is>
+      <x:c r="G3" s="31" t="str">
+        <x:v>Functional provisional implementation; design review and approval still required. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -9964,10 +9960,8 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G4" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Approved/coded; needs machine playtest and polish.</x:t>
-        </x:is>
+      <x:c r="G4" s="31" t="str">
+        <x:v>Approved/coded; needs machine playtest and polish. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -9999,10 +9993,8 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G5" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Functional provisional implementation; design review and approval still required.</x:t>
-        </x:is>
+      <x:c r="G5" s="31" t="str">
+        <x:v>Functional provisional implementation; design review and approval still required. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="132" hidden="0" customHeight="1">
@@ -10033,7 +10025,7 @@
         <x:v>No individual Case File powers. Each 1X phase Jackpot = 100K + 20K × the chapter's collected Case Files (0–25 files; +0–500K). 2X phase Jackpots double both base and prep. The rooftop Super is separate at 1M × successful phases and does not receive Wizard Prep.</x:v>
       </x:c>
       <x:c r="G6" s="31" t="str">
-        <x:v>Approved/coded from the 2026-09-01 design: repeating 2-ball/VUK-lock wizard with Fiddler, Metal-Eating Monster, Conquistador, Spider-Slayer, and Harley &amp; Clivendon phases; saucers park excess balls; Chapter Case Files add 20K to every 1X phase JP; phase wins build a 1M-per-success rooftop Super. Needs machine playtest and polish. Fiddler parity update: both drop banks stage down during GET READY; individual drop switches are ignored; the exposed left/right bank rubbers are the bank-note inputs; WATCH strobe, note gaps, repeat pause, and correct/wrong feedback match standalone Fiddler.</x:v>
+        <x:v>Approved/coded from the 2026-09-01 design: repeating 2-ball/VUK-lock wizard with Fiddler, Metal-Eating Monster, Conquistador, Spider-Slayer, and Harley &amp; Clivendon phases; saucers park excess balls; Chapter Case Files add 20K to every 1X phase JP; phase wins build a 1M-per-success rooftop Super. Needs machine playtest and polish. Fiddler parity update: both drop banks stage down during GET READY; individual drop switches are ignored; the exposed left/right bank rubbers are the bank-note inputs; WATCH strobe, note gaps, repeat pause, and correct/wrong feedback match standalone Fiddler. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10066,7 +10058,7 @@
         </x:is>
       </x:c>
       <x:c r="G7" s="31" t="str">
-        <x:v>Functional provisional implementation; design review and approval still required. Recent VUK timing fix: active gameplay VUK visits use the shared 1.5-second delayed release for both unlit and Curse Jackpot shots; the post-introduction launch remains immediate. Physical timing needs playtest.</x:v>
+        <x:v>Functional provisional implementation; design review and approval still required. Recent VUK timing fix: active gameplay VUK visits use the shared 1.5-second delayed release for both unlit and Curse Jackpot shots; the post-introduction launch remains immediate. Physical timing needs playtest. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10097,7 +10089,7 @@
         <x:v>No individual Case File powers. Every Gas and Noah Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Red/yellow gas awards, upper-spinner build increments, and the 1M four-ball Magneto award do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G8" s="31" t="str">
-        <x:v>Approved/coded: repeating 3-ball multiball with 20s opening save. Each left drop releases one independent gas zone; lower-spinner hits cool all active zones red → yellow → green; green collects a 500K+ Case File Gas Jackpot. Upper targets and early right-drop hits eliminate Noah's false locations; the last standing right target collects a 500K+ Case File + 100K-per-upper-spin Noah Jackpot. Saucers park up to two balls for 2X/3X Noah and release on collect. Middle A+B lights center web for 10s: Add-a-Ball with 10s save below four balls, otherwise 1M. No final objective; ends when multiball ends. Needs machine playtest and presentation polish.</x:v>
+        <x:v>Approved/coded: repeating 3-ball multiball with 20s opening save. Each left drop releases one independent gas zone; lower-spinner hits cool all active zones red → yellow → green; green collects a 500K+ Case File Gas Jackpot. Upper targets and early right-drop hits eliminate Noah's false locations; the last standing right target collects a 500K+ Case File + 100K-per-upper-spin Noah Jackpot. Saucers park up to two balls for 2X/3X Noah and release on collect. Middle A+B lights center web for 10s: Add-a-Ball with 10s save below four balls, otherwise 1M. No final objective; ends when multiball ends. Needs machine playtest and presentation polish. Ordinary parking: 12s.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10130,7 +10122,7 @@
         </x:is>
       </x:c>
       <x:c r="G9" s="31" t="str">
-        <x:v>Implemented repeating elemental-chain multiball; Blotto attack now accumulates up to three simultaneous solid-purple blocked zones during the thaw stage, with attack cadence 8s / 7s / 6s by cycle. Star clears all blocked zones and resets the timer. Needs machine playtest/polish.</x:v>
+        <x:v>Implemented repeating elemental-chain multiball; Blotto attack now accumulates up to three simultaneous solid-purple blocked zones during the thaw stage, with attack cadence 8s / 7s / 6s by cycle. Star clears all blocked zones and resets the timer. Needs machine playtest/polish. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10163,7 +10155,7 @@
         </x:is>
       </x:c>
       <x:c r="G10" s="31" t="str">
-        <x:v>Implemented 3-ball VUK/saucer relay wizard cycling Igor, Molemen, and DeVargas lower phases into escalating Doctor Atlantean rooftop jackpots; needs machine playtest/polish.</x:v>
+        <x:v>Implemented 3-ball VUK/saucer relay wizard cycling Igor, Molemen, and DeVargas lower phases into escalating Doctor Atlantean rooftop jackpots; needs machine playtest/polish. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10196,7 +10188,7 @@
         </x:is>
       </x:c>
       <x:c r="G11" s="31" t="str">
-        <x:v>Implemented repeating 2-ball investigation multiball: hit both pops to reveal one random no-repeat Cameo pair (A/B, slings, or bank rubbers); rubber pair is exposed one bank drop per upper-spinner spin. Any flashing saucer reveals the correct Cameo target; early candidate hits score 100K with Daily Bugle impostor audio; correct Cameo scores 1M + Case Files. Desperado requires all five unique right drops at 50K with bank reset after every hit and upper-spinner spotting. Brutus lights all three saucers; left-bank hit closes them, right-bank hit relights them; any lit saucer scores 500K + Case Files. Then gate opens for a 20s 2M + Case Files VUK Super; collect or miss returns to Cameo. Global upper L/C/R completion adds a ball to a four-ball max with 15s save, or 500K + Case Files at cap. Needs machine playtest/polish.</x:v>
+        <x:v>Implemented repeating 2-ball investigation multiball: hit both pops to reveal one random no-repeat Cameo pair (A/B, slings, or bank rubbers); rubber pair is exposed one bank drop per upper-spinner spin. Any flashing saucer reveals the correct Cameo target; early candidate hits score 100K with Daily Bugle impostor audio; correct Cameo scores 1M + Case Files. Desperado requires all five unique right drops at 50K with bank reset after every hit and upper-spinner spotting. Brutus lights all three saucers; left-bank hit closes them, right-bank hit relights them; any lit saucer scores 500K + Case Files. Then gate opens for a 20s 2M + Case Files VUK Super; collect or miss returns to Cameo. Global upper L/C/R completion adds a ball to a four-ball max with 15s save, or 500K + Case Files at cap. Needs machine playtest/polish. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -10227,7 +10219,7 @@
         <x:v>Wizard scoring uses Chapter 11 Case Files directly: Master Vine targets = 100K + 20K × collected Case Files; Spider-Men lit-position Jackpots = 250K + 20K × collected Case Files; Master Technician spinner/Star-at-cap = 100K + 20K × collected Case Files + 10K × rooftop upper-target hits. Rooftop setup shots themselves receive only normal/basic upper-playfield scoring.</x:v>
       </x:c>
       <x:c r="G12" s="31" t="str">
-        <x:v>Implemented endurance wizard: 3-ball multiball, 20s opening save, 4-ball cap. Each rooftop visit gives 12 setup flips; upper targets build Master Technician value and qualify Spider-Men saucers, while upper-spinner spins light Master Vine shots. Exit selects the lower phase (L Spider-Men / C Master Vine / R Master Technician). Gate opens only for rooftop setup, saucers park for 15s, and the loop repeats until multiball ends. Needs machine playtest/polish.</x:v>
+        <x:v>Implemented endurance wizard: 3-ball multiball, 20s opening save, 4-ball cap. Each rooftop visit gives 12 setup flips; upper targets build Master Technician value and qualify Spider-Men saucers, while upper-spinner spins light Master Vine shots. Exit selects the lower phase (L Spider-Men / C Master Vine / R Master Technician). Gate opens only for rooftop setup, saucers park for 12s, and the loop repeats until multiball ends. Needs machine playtest/polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10261,10 +10253,8 @@
           <x:t xml:space="preserve">Separate final wizard after all 11 chapter wizards.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G13" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Working generic framework; dedicated Kingpin design/retheme remains unfinished.</x:t>
-        </x:is>
+      <x:c r="G13" s="31" t="str">
+        <x:v>Working generic framework; dedicated Kingpin design/retheme remains unfinished. Timing: 12s ordinary parking; 20s opening ball save.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>